<commit_message>
chore: update project files
</commit_message>
<xml_diff>
--- a/Multiarray_Extracts/Vapp_Analysis.xlsx
+++ b/Multiarray_Extracts/Vapp_Analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8061bcffd0d95ffa/Desktop/WAVEGIUDE HELPERS/6by6array/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8061bcffd0d95ffa/Desktop/UNIVERSITY/S1 2026/EGH490-2/Multiarray_Extracts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="775" documentId="8_{8523630A-D4FD-420B-B44C-C824167AD9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{905C701D-5426-41A5-B5D2-5CB93E6C60C8}"/>
+  <xr:revisionPtr revIDLastSave="777" documentId="8_{8523630A-D4FD-420B-B44C-C824167AD9C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4344AF17-6771-421D-B6DA-A07F193E4A4A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E4EEB7EC-7293-42E9-9FCB-F1798A8A708C}"/>
   </bookViews>
@@ -1140,26 +1140,71 @@
     <xf numFmtId="168" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1188,71 +1233,26 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="10" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="10" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1271,1126 +1271,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="1F3864"/>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman"/>
-                <a:ea typeface="Times New Roman"/>
-                <a:cs typeface="Times New Roman"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Error Surface: Normalized |Vapp| − Target</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="1F3864"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:ea typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:view3D>
-      <c:rotX val="15"/>
-      <c:rotY val="20"/>
-      <c:rAngAx val="0"/>
-    </c:view3D>
-    <c:floor>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:floor>
-    <c:sideWall>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:sideWall>
-    <c:backWall>
-      <c:thickness val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-        <a:sp3d/>
-      </c:spPr>
-    </c:backWall>
-    <c:plotArea>
-      <c:layout/>
-      <c:surface3DChart>
-        <c:wireframe val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$53</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>i \ j</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$53:$G$53</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>6</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$54</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$54:$G$54</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000;\-0.0000;0.0000</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>1.8527878705346057E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>-1.3710411620572405E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.6131629597342831E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>-1.8664756863358112E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.4986737642380898E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>-2.3841362288676282E-4</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$55</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>2</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$55:$G$55</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000;\-0.0000;0.0000</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>3.7881617507562859E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3.6041254885529783E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3.987906719181189E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4.6511281466689369E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3.5978848476875158E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3.5898963663262007E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$56</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>3</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$56:$G$56</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000;\-0.0000;0.0000</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>2.6243720754504596E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.9293308316743536E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-2.7398756939976621E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>-4.7688633481985931E-3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>-6.2026110084655306E-3</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3.8013191703876903E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$57</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>4</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent5"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$57:$G$57</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000;\-0.0000;0.0000</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>4.3947592185135276E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>8.1868647562708396E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.8000139882706998E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4.1674804054678827E-3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3.0103644662959117E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3.2330214317713213E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'CurveRad Vapp'!$A$58</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>5</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent6"/>
-            </a:solidFill>
-            <a:ln/>
-            <a:effectLst/>
-            <a:sp3d/>
-          </c:spPr>
-          <c:cat>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$52:$G$52</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'CurveRad Vapp'!$B$58:$G$58</c:f>
-              <c:numCache>
-                <c:formatCode>0.0000;\-0.0000;0.0000</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>2.852590139213762E-2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2.1086792150757039E-2</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.0355845301145981E-2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.7104605231316183E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>2.4481849460246008E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3.4505204149830881E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-AF4D-4FFC-B62B-DF16C5D82955}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:bandFmts>
-          <c:bandFmt>
-            <c:idx val="0"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="1"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="2"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="3"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="4"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="6"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="7"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="8"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="9"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="10"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="11"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent6">
-                  <a:lumMod val="60000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="12"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="13"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-          <c:bandFmt>
-            <c:idx val="14"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent3">
-                  <a:lumMod val="80000"/>
-                  <a:lumOff val="20000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:ln/>
-              <a:effectLst/>
-              <a:sp3d/>
-            </c:spPr>
-          </c:bandFmt>
-        </c:bandFmts>
-        <c:axId val="1968089647"/>
-        <c:axId val="1968084367"/>
-        <c:axId val="1495249119"/>
-      </c:surface3DChart>
-      <c:catAx>
-        <c:axId val="1968089647"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="Times New Roman"/>
-                    <a:ea typeface="Times New Roman"/>
-                    <a:cs typeface="Times New Roman"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>j (column index)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman"/>
-                  <a:ea typeface="Times New Roman"/>
-                  <a:cs typeface="Times New Roman"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman"/>
-                <a:ea typeface="Times New Roman"/>
-                <a:cs typeface="Times New Roman"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1968084367"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1968084367"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="Times New Roman"/>
-                    <a:ea typeface="Times New Roman"/>
-                    <a:cs typeface="Times New Roman"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Error</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman"/>
-                  <a:ea typeface="Times New Roman"/>
-                  <a:cs typeface="Times New Roman"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman"/>
-                <a:ea typeface="Times New Roman"/>
-                <a:cs typeface="Times New Roman"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1968089647"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:serAx>
-        <c:axId val="1495249119"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="Times New Roman"/>
-                    <a:ea typeface="Times New Roman"/>
-                    <a:cs typeface="Times New Roman"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-AU"/>
-                  <a:t>i (row index)</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman"/>
-                  <a:ea typeface="Times New Roman"/>
-                  <a:cs typeface="Times New Roman"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman"/>
-                <a:ea typeface="Times New Roman"/>
-                <a:cs typeface="Times New Roman"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1968084367"/>
-        <c:crosses val="autoZero"/>
-      </c:serAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr rtl="0">
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:ea typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="zero"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:srgbClr val="BFBFBF"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>217237</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>116974</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>344237</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>86896</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3AB6199D-973B-E93E-2D90-CBAF72CA65A8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2725,45 +1607,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="28" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="I1" s="46" t="s">
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="I1" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="Q1" s="47" t="s">
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="Q1" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
-      <c r="W1" s="49"/>
+      <c r="R1" s="79"/>
+      <c r="S1" s="79"/>
+      <c r="T1" s="79"/>
+      <c r="U1" s="79"/>
+      <c r="V1" s="79"/>
+      <c r="W1" s="80"/>
     </row>
     <row r="2" spans="1:23" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="Q2" s="65">
+      <c r="Q2" s="49">
         <f>AVERAGE(D16,E16,D17,E17)</f>
         <v>10.774734390529215</v>
       </c>
-      <c r="R2" s="66"/>
-      <c r="S2" s="66"/>
-      <c r="T2" s="66"/>
-      <c r="U2" s="66"/>
-      <c r="V2" s="66"/>
-      <c r="W2" s="67"/>
+      <c r="R2" s="50"/>
+      <c r="S2" s="50"/>
+      <c r="T2" s="50"/>
+      <c r="U2" s="50"/>
+      <c r="V2" s="50"/>
+      <c r="W2" s="51"/>
     </row>
     <row r="3" spans="1:23" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="13" t="s">
@@ -2808,15 +1690,15 @@
       <c r="O3" s="19">
         <v>6</v>
       </c>
-      <c r="Q3" s="68" t="s">
+      <c r="Q3" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
-      <c r="T3" s="69"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="69"/>
-      <c r="W3" s="70"/>
+      <c r="R3" s="53"/>
+      <c r="S3" s="53"/>
+      <c r="T3" s="53"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="54"/>
     </row>
     <row r="4" spans="1:23" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="23">
@@ -2905,15 +1787,15 @@
       <c r="O5" s="15">
         <v>-2.1609317611943002</v>
       </c>
-      <c r="Q5" s="71" t="s">
+      <c r="Q5" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="R5" s="72"/>
-      <c r="S5" s="72"/>
-      <c r="T5" s="72"/>
-      <c r="U5" s="72"/>
-      <c r="V5" s="72"/>
-      <c r="W5" s="73"/>
+      <c r="R5" s="56"/>
+      <c r="S5" s="56"/>
+      <c r="T5" s="56"/>
+      <c r="U5" s="56"/>
+      <c r="V5" s="56"/>
+      <c r="W5" s="57"/>
     </row>
     <row r="6" spans="1:23" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="24">
@@ -2958,16 +1840,16 @@
       <c r="O6" s="15">
         <v>-2.6174743859838001</v>
       </c>
-      <c r="Q6" s="74">
+      <c r="Q6" s="58">
         <f>AVERAGE(D26,E26,D27,E27)</f>
         <v>-49.875224363557706</v>
       </c>
-      <c r="R6" s="75"/>
-      <c r="S6" s="75"/>
-      <c r="T6" s="75"/>
-      <c r="U6" s="75"/>
-      <c r="V6" s="75"/>
-      <c r="W6" s="76"/>
+      <c r="R6" s="59"/>
+      <c r="S6" s="59"/>
+      <c r="T6" s="59"/>
+      <c r="U6" s="59"/>
+      <c r="V6" s="59"/>
+      <c r="W6" s="60"/>
     </row>
     <row r="7" spans="1:23" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="24">
@@ -3012,15 +1894,15 @@
       <c r="O7" s="15">
         <v>-2.7236335369845999</v>
       </c>
-      <c r="Q7" s="77" t="s">
+      <c r="Q7" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="R7" s="78"/>
-      <c r="S7" s="78"/>
-      <c r="T7" s="78"/>
-      <c r="U7" s="78"/>
-      <c r="V7" s="78"/>
-      <c r="W7" s="79"/>
+      <c r="R7" s="62"/>
+      <c r="S7" s="62"/>
+      <c r="T7" s="62"/>
+      <c r="U7" s="62"/>
+      <c r="V7" s="62"/>
+      <c r="W7" s="63"/>
     </row>
     <row r="8" spans="1:23" ht="20" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="24">
@@ -3109,68 +1991,68 @@
       <c r="O9" s="16">
         <v>-1.1965266421292999</v>
       </c>
-      <c r="Q9" s="80" t="s">
+      <c r="Q9" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="R9" s="81"/>
-      <c r="S9" s="81"/>
-      <c r="T9" s="81"/>
-      <c r="U9" s="81"/>
-      <c r="V9" s="81"/>
-      <c r="W9" s="82"/>
+      <c r="R9" s="65"/>
+      <c r="S9" s="65"/>
+      <c r="T9" s="65"/>
+      <c r="U9" s="65"/>
+      <c r="V9" s="65"/>
+      <c r="W9" s="66"/>
     </row>
     <row r="10" spans="1:23" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="Q10" s="52" t="s">
+      <c r="Q10" s="67" t="s">
         <v>17</v>
       </c>
-      <c r="R10" s="53"/>
-      <c r="S10" s="53"/>
-      <c r="T10" s="53"/>
-      <c r="U10" s="53"/>
-      <c r="V10" s="53"/>
-      <c r="W10" s="54"/>
+      <c r="R10" s="68"/>
+      <c r="S10" s="68"/>
+      <c r="T10" s="68"/>
+      <c r="U10" s="68"/>
+      <c r="V10" s="68"/>
+      <c r="W10" s="69"/>
     </row>
     <row r="11" spans="1:23" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="50" t="s">
+      <c r="A11" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="50"/>
-      <c r="I11" s="51" t="s">
+      <c r="B11" s="81"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="81"/>
+      <c r="G11" s="81"/>
+      <c r="I11" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="J11" s="51"/>
-      <c r="K11" s="51"/>
-      <c r="L11" s="51"/>
-      <c r="M11" s="51"/>
-      <c r="N11" s="51"/>
-      <c r="O11" s="51"/>
-      <c r="Q11" s="52" t="str">
+      <c r="J11" s="82"/>
+      <c r="K11" s="82"/>
+      <c r="L11" s="82"/>
+      <c r="M11" s="82"/>
+      <c r="N11" s="82"/>
+      <c r="O11" s="82"/>
+      <c r="Q11" s="67" t="str">
         <f>"Phase deviation at (3,3), (3,4), (4,3), (4,4) = "&amp;TEXT(L36,"0.00")&amp;"°, "&amp;TEXT(M36,"0.00")&amp;"°, "&amp;TEXT(L37,"0.00")&amp;"°, "&amp;TEXT(M37,"0.00")&amp;"°  (all drift around 0°)"</f>
         <v>Phase deviation at (3,3), (3,4), (4,3), (4,4) = 1.78°, -0.55°, -1.50°, 0.27°  (all drift around 0°)</v>
       </c>
-      <c r="R11" s="53"/>
-      <c r="S11" s="53"/>
-      <c r="T11" s="53"/>
-      <c r="U11" s="53"/>
-      <c r="V11" s="53"/>
-      <c r="W11" s="54"/>
+      <c r="R11" s="68"/>
+      <c r="S11" s="68"/>
+      <c r="T11" s="68"/>
+      <c r="U11" s="68"/>
+      <c r="V11" s="68"/>
+      <c r="W11" s="69"/>
     </row>
     <row r="12" spans="1:23" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="Q12" s="61" t="str" cm="1">
+      <c r="Q12" s="45" t="str" cm="1">
         <f t="array" ref="Q12">"Error vs target: max |error| = "&amp;TEXT(MAX(ABS(B54:G59)),"0.0000")&amp;",  RMS = "&amp;TEXT(SQRT(SUMPRODUCT(B54:G59,B54:G59)/36),"0.0000")</f>
         <v>Error vs target: max |error| = 0.0465,  RMS = 0.0262</v>
       </c>
-      <c r="R12" s="62"/>
-      <c r="S12" s="62"/>
-      <c r="T12" s="62"/>
-      <c r="U12" s="62"/>
-      <c r="V12" s="62"/>
-      <c r="W12" s="63"/>
+      <c r="R12" s="46"/>
+      <c r="S12" s="46"/>
+      <c r="T12" s="46"/>
+      <c r="U12" s="46"/>
+      <c r="V12" s="46"/>
+      <c r="W12" s="47"/>
     </row>
     <row r="13" spans="1:23" ht="22" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A13" s="29" t="s">
@@ -3554,24 +2436,24 @@
     </row>
     <row r="20" spans="1:15" ht="38" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="58" t="s">
+      <c r="A21" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="58"/>
-      <c r="C21" s="58"/>
-      <c r="D21" s="58"/>
-      <c r="E21" s="58"/>
-      <c r="F21" s="58"/>
-      <c r="G21" s="58"/>
-      <c r="I21" s="59" t="s">
+      <c r="B21" s="73"/>
+      <c r="C21" s="73"/>
+      <c r="D21" s="73"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="73"/>
+      <c r="G21" s="73"/>
+      <c r="I21" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="J21" s="59"/>
-      <c r="K21" s="59"/>
-      <c r="L21" s="59"/>
-      <c r="M21" s="59"/>
-      <c r="N21" s="59"/>
-      <c r="O21" s="59"/>
+      <c r="J21" s="74"/>
+      <c r="K21" s="74"/>
+      <c r="L21" s="74"/>
+      <c r="M21" s="74"/>
+      <c r="N21" s="74"/>
+      <c r="O21" s="74"/>
     </row>
     <row r="22" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="23" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -3956,24 +2838,24 @@
     </row>
     <row r="30" spans="1:15" ht="38.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="31" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="60" t="s">
+      <c r="A31" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="60"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="60"/>
-      <c r="I31" s="64" t="s">
+      <c r="B31" s="75"/>
+      <c r="C31" s="75"/>
+      <c r="D31" s="75"/>
+      <c r="E31" s="75"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="I31" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="J31" s="64"/>
-      <c r="K31" s="64"/>
-      <c r="L31" s="64"/>
-      <c r="M31" s="64"/>
-      <c r="N31" s="64"/>
-      <c r="O31" s="64"/>
+      <c r="J31" s="48"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="48"/>
+      <c r="M31" s="48"/>
+      <c r="N31" s="48"/>
+      <c r="O31" s="48"/>
     </row>
     <row r="32" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="33" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -4358,24 +3240,24 @@
     </row>
     <row r="40" spans="1:15" ht="38.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="41" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="55" t="s">
+      <c r="A41" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="B41" s="55"/>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="55"/>
-      <c r="I41" s="57" t="s">
+      <c r="B41" s="70"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="70"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="70"/>
+      <c r="I41" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="J41" s="57"/>
-      <c r="K41" s="57"/>
-      <c r="L41" s="57"/>
-      <c r="M41" s="57"/>
-      <c r="N41" s="57"/>
-      <c r="O41" s="57"/>
+      <c r="J41" s="72"/>
+      <c r="K41" s="72"/>
+      <c r="L41" s="72"/>
+      <c r="M41" s="72"/>
+      <c r="N41" s="72"/>
+      <c r="O41" s="72"/>
     </row>
     <row r="42" spans="1:15" ht="6.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="43" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -4724,15 +3606,15 @@
     </row>
     <row r="50" spans="1:15" ht="36.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="51" spans="1:15" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="56" t="s">
+      <c r="A51" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="B51" s="56"/>
-      <c r="C51" s="56"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="56"/>
+      <c r="B51" s="71"/>
+      <c r="C51" s="71"/>
+      <c r="D51" s="71"/>
+      <c r="E51" s="71"/>
+      <c r="F51" s="71"/>
+      <c r="G51" s="71"/>
     </row>
     <row r="52" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="53" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -4945,6 +3827,18 @@
     <row r="70" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I1:O1"/>
+    <mergeCell ref="Q1:W1"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="I11:O11"/>
+    <mergeCell ref="Q11:W11"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="I41:O41"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="I21:O21"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="Q12:W12"/>
     <mergeCell ref="I31:O31"/>
     <mergeCell ref="Q2:W2"/>
@@ -4954,18 +3848,6 @@
     <mergeCell ref="Q7:W7"/>
     <mergeCell ref="Q9:W9"/>
     <mergeCell ref="Q10:W10"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A51:G51"/>
-    <mergeCell ref="I41:O41"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="I21:O21"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="I1:O1"/>
-    <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="I11:O11"/>
-    <mergeCell ref="Q11:W11"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:G9">
     <cfRule type="colorScale" priority="1">
@@ -5086,6 +3968,5 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>